<commit_message>
running specific tests to debug on ci
</commit_message>
<xml_diff>
--- a/yt_multi_language_ui_validator/src/main/resources/data/ApplicableLanguageExpectedLanguage.xlsx
+++ b/yt_multi_language_ui_validator/src/main/resources/data/ApplicableLanguageExpectedLanguage.xlsx
@@ -453,7 +453,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CROATIAN</t>
+          <t>BOSNIAN</t>
         </is>
       </c>
     </row>
@@ -753,7 +753,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>SLOVENIAN</t>
+          <t>SLOVENE</t>
         </is>
       </c>
     </row>
@@ -933,7 +933,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>BANGLA</t>
+          <t>BENGALI</t>
         </is>
       </c>
     </row>

</xml_diff>